<commit_message>
Expand workbook, skills, and add Odoo seeding script
- Rewrite odoo-skill-workbook.md and README with expanded exercises
- Update the three example skills with fuller procedures
- Add materials/seed/seed_workshop_data.py for pre-workshop Odoo setup
- Point .mcp.json at the workshop Odoo instance

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/materials/신규협력사.xlsx
+++ b/materials/신규협력사.xlsx
@@ -39,8 +39,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004472C4"/>
-        <bgColor rgb="004472C4"/>
+        <fgColor rgb="004A5568"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +58,7 @@
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,11 +425,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
@@ -460,110 +459,124 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SUP-03 정밀가공(주)</t>
+          <t>(주)태성정공</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>contact@sup03-precision.co.kr</t>
+          <t>sales@taesung-machine.example.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>02-1234-5601</t>
+          <t>031-555-1101</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>김정밀</t>
+          <t>오세훈</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SUP-04 케이블어셈블리</t>
+          <t>유진하이테크(주)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>sales@sup04-cable.co.kr</t>
+          <t>info@eugene-hitech.example.com</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>02-1234-5602</t>
+          <t>043-555-1202</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>이케이블</t>
+          <t>배정민</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SUP-05 표면처리기술</t>
+          <t>(주)정우정밀</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>info@sup05-surface.co.kr</t>
+          <t>order@jw-precision.example.com</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>031-987-6503</t>
+          <t>031-555-0303</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>박표면</t>
+          <t>이준호</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SUP-06 금형센터</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>biz@sup06-mold.co.kr</t>
-        </is>
-      </c>
+          <t>남광열처리</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
-          <t>032-555-7704</t>
+          <t>052-555-1404</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>최금형</t>
+          <t>서지훈</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>SUP-07 물류파트너스</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
-          <t>cs@sup07-logistics.co.kr</t>
+          <t>ghost@example.com</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>010-2222-8805</t>
+          <t>02-555-1505</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>정물류</t>
+          <t>미상</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>대성EMC(주)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>contact@daesung-emc.example.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>031-555-1606</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>윤하늘</t>
         </is>
       </c>
     </row>

</xml_diff>